<commit_message>
Added the ability to get excel worksheets by name
</commit_message>
<xml_diff>
--- a/src/Root16.Sprout.Excel.Sample/Data/test.xlsx
+++ b/src/Root16.Sprout.Excel.Sample/Data/test.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JohnPeters\source\repos\Root16\sprout\src\Root16.Sprout.Excel.Sample\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repos\Root16\sprout\src\Root16.Sprout.Excel.Sample\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{874F0B8A-8BE9-43A6-B065-4A561E1592F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{565DAAF3-8DE4-43C3-A34A-B6EE401E6881}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{CEB87106-A47A-4C98-9558-1BFE9B2A2111}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" activeTab="2" xr2:uid="{CEB87106-A47A-4C98-9558-1BFE9B2A2111}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="ExampleSheet" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="16">
   <si>
     <t>Account Name</t>
   </si>
@@ -457,16 +458,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80BB2943-661C-4C64-9509-0DD82479A2B9}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.44140625" customWidth="1"/>
-    <col min="4" max="4" width="22.109375" customWidth="1"/>
-    <col min="5" max="5" width="25.77734375" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.42578125" customWidth="1"/>
+    <col min="4" max="4" width="22.140625" customWidth="1"/>
+    <col min="5" max="5" width="25.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>11</v>
       </c>
@@ -483,7 +484,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -500,7 +501,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -517,7 +518,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -543,16 +544,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CB80B9F-6FD1-475B-9E6A-A17FA4DA8102}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.33203125" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" customWidth="1"/>
-    <col min="3" max="3" width="16.33203125" customWidth="1"/>
-    <col min="4" max="4" width="17.6640625" customWidth="1"/>
-    <col min="5" max="5" width="22.44140625" customWidth="1"/>
+    <col min="1" max="1" width="25.28515625" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" customWidth="1"/>
+    <col min="5" max="5" width="22.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -569,7 +570,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -589,4 +590,90 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{722DC654-A4BA-4077-9FA3-948ECB282307}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.42578125" customWidth="1"/>
+    <col min="4" max="4" width="22.140625" customWidth="1"/>
+    <col min="5" max="5" width="25.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2">
+        <v>-0.05</v>
+      </c>
+      <c r="D2">
+        <v>17.777000000000001</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>83.25</v>
+      </c>
+      <c r="D3">
+        <v>17.777000000000001</v>
+      </c>
+      <c r="E3">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4">
+        <v>0.222222</v>
+      </c>
+      <c r="D4">
+        <v>17.777000000000001</v>
+      </c>
+      <c r="E4">
+        <v>-25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>